<commit_message>
fix(backend): update requirements for python 3.14 and configure pyre2 paths
</commit_message>
<xml_diff>
--- a/PILi_Quarts_V4.0_Studio/backend/modules/N04_Binary_Factory/output_sandbox/STUDIO_COTIZACION_SIMPLE.xlsx
+++ b/PILi_Quarts_V4.0_Studio/backend/modules/N04_Binary_Factory/output_sandbox/STUDIO_COTIZACION_SIMPLE.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;S/&quot; #,##0.00"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -33,13 +33,13 @@
       <sz val="9"/>
     </font>
     <font>
-      <color rgb="00A855F7"/>
+      <color rgb="0022C55E"/>
       <sz val="8"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00A855F7"/>
+      <color rgb="0022C55E"/>
       <sz val="18"/>
     </font>
     <font>
@@ -50,12 +50,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00A855F7"/>
+      <color rgb="0022C55E"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00A855F7"/>
+      <color rgb="0022C55E"/>
       <sz val="12"/>
       <u val="single"/>
     </font>
@@ -67,7 +67,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00A855F7"/>
+      <color rgb="0022C55E"/>
     </font>
     <font>
       <b val="1"/>
@@ -86,7 +86,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -95,14 +95,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00A855F7"/>
-        <bgColor rgb="00A855F7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F9FAFB"/>
-        <bgColor rgb="00F9FAFB"/>
+        <fgColor rgb="0022C55E"/>
+        <bgColor rgb="0022C55E"/>
       </patternFill>
     </fill>
   </fills>
@@ -132,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -154,16 +148,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -258,12 +242,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>0</col>
+      <col>1</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1714500" cy="571500"/>
+    <ext cx="571500" cy="571500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -573,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -709,190 +693,60 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="n">
-        <v>450</v>
-      </c>
-      <c r="F15" s="11" t="n">
-        <v>450</v>
-      </c>
-    </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>cto</t>
-        </is>
-      </c>
-      <c r="E16" s="14" t="n">
-        <v>120</v>
-      </c>
-      <c r="F16" s="14" t="n">
-        <v>720</v>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>SUBTOTAL:</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="n">
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>IGV (18%):</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>pto</t>
-        </is>
-      </c>
-      <c r="E17" s="11" t="n">
-        <v>45</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>450</v>
-      </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>pto</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="n">
-        <v>35</v>
-      </c>
-      <c r="F18" s="14" t="n">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>glb</t>
-        </is>
-      </c>
-      <c r="E19" s="11" t="n">
-        <v>850</v>
-      </c>
-      <c r="F19" s="11" t="n">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="D21" s="15" t="inlineStr">
-        <is>
-          <t>SUBTOTAL:</t>
-        </is>
-      </c>
-      <c r="F21" s="16" t="n">
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL:</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="22">
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>IGV (18%):</t>
-        </is>
-      </c>
-      <c r="F22" s="16" t="n">
-        <v>10</v>
-      </c>
-    </row>
+    <row r="22"/>
     <row r="23">
-      <c r="D23" s="17" t="inlineStr">
-        <is>
-          <t>TOTAL:</t>
-        </is>
-      </c>
-      <c r="F23" s="18" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="19" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>TESLA ELECTRICIDAD Y AUTOMATIZACIÓN S.A.C.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="20" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>RUC: 20601138787 | Teléfono: 906 315 961</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="20" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>Email: ingenieria.teslaelectricidad@gmail.com</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="20" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Jr. Las Ágatas Mz B Lote 09, Urb. San Carlos, SJL</t>
         </is>
@@ -902,26 +756,26 @@
   <mergeCells count="22">
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A23:F23"/>
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="D8:F8"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="D17:E17"/>
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="D16:E16"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="D1:F3"/>
-    <mergeCell ref="A31:F31"/>
     <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="A22:E22"/>
     <mergeCell ref="D10:F10"/>
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D23:E23"/>
     <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>